<commit_message>
Day 3 : adding feature file and pages(page factory) for 'Buy Medicine' Module --- Arpan Mitra
</commit_message>
<xml_diff>
--- a/Manual_Testing/Arpan_Mitra_Apollo_247_Buy_Medicines.xlsx
+++ b/Manual_Testing/Arpan_Mitra_Apollo_247_Buy_Medicines.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Capgemini Training\Sprint Implementation\CG_Sprint_GRP_6_Testing\Day_1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Capgemini Training\Sprint Implementation\Sprint_GROUP_6_Testing\Manual_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D85BFC1-D824-4374-A202-216E3760E6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7D4C13-8533-4F1D-B311-4D120677A593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{F3877DBE-F13B-4A1F-AFB6-72D4C9E72E87}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{F3877DBE-F13B-4A1F-AFB6-72D4C9E72E87}"/>
   </bookViews>
   <sheets>
     <sheet name="User Story" sheetId="1" r:id="rId1"/>
@@ -1142,7 +1142,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1235,89 +1235,52 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2814,7 +2777,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D6" s="45"/>
+      <c r="D6" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2835,7 +2798,7 @@
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="16.36328125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="14.6328125" style="36" customWidth="1"/>
+    <col min="5" max="5" width="14.6328125" customWidth="1"/>
     <col min="6" max="6" width="19.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2852,27 +2815,27 @@
       <c r="D1" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="34" t="s">
         <v>203</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="36" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="42" t="s">
         <v>206</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="42" t="s">
         <v>205</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="42" t="s">
         <v>105</v>
       </c>
       <c r="D2" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F2" s="19" t="s">
@@ -2880,13 +2843,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="34"/>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
+      <c r="A3" s="42"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
       <c r="D3" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="35" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="19" t="s">
@@ -2894,13 +2857,13 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
+      <c r="A4" s="42"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
       <c r="D4" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E4" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F4" s="19" t="s">
@@ -2920,7 +2883,7 @@
       <c r="D5" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F5" s="19" t="s">
@@ -2928,19 +2891,19 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="42" t="s">
         <v>208</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="42" t="s">
         <v>110</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="39" t="s">
+      <c r="E6" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F6" s="19" t="s">
@@ -2948,13 +2911,13 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="34"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="34"/>
+      <c r="A7" s="42"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
       <c r="D7" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="39" t="s">
+      <c r="E7" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F7" s="19" t="s">
@@ -2962,19 +2925,19 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="42" t="s">
         <v>216</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="42" t="s">
         <v>112</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="39" t="s">
+      <c r="E8" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F8" s="19" t="s">
@@ -2982,13 +2945,13 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="34"/>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
       <c r="D9" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="39" t="s">
+      <c r="E9" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F9" s="19" t="s">
@@ -2996,19 +2959,19 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="42" t="s">
         <v>217</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="42" t="s">
         <v>210</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="42" t="s">
         <v>114</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="19" t="s">
@@ -3016,13 +2979,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="34"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
       <c r="D11" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F11" s="19" t="s">
@@ -3030,19 +2993,19 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="42" t="s">
         <v>211</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="42" t="s">
         <v>116</v>
       </c>
       <c r="D12" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F12" s="19" t="s">
@@ -3050,13 +3013,13 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="34"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
       <c r="D13" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F13" s="19" t="s">
@@ -3064,13 +3027,13 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="34"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
       <c r="D14" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F14" s="19" t="s">
@@ -3090,7 +3053,7 @@
       <c r="D15" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="39" t="s">
+      <c r="E15" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F15" s="19" t="s">
@@ -3098,19 +3061,19 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="42" t="s">
         <v>219</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="42" t="s">
         <v>213</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="42" t="s">
         <v>181</v>
       </c>
       <c r="D16" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="39" t="s">
+      <c r="E16" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F16" s="19" t="s">
@@ -3118,13 +3081,13 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="34"/>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
       <c r="D17" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="E17" s="39" t="s">
+      <c r="E17" s="47" t="s">
         <v>65</v>
       </c>
       <c r="F17" s="19" t="s">
@@ -3132,19 +3095,19 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="34" t="s">
+      <c r="A18" s="42" t="s">
         <v>249</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="42" t="s">
         <v>250</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="42" t="s">
         <v>234</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="E18" s="37" t="s">
+      <c r="E18" s="44" t="s">
         <v>70</v>
       </c>
       <c r="F18" s="46" t="s">
@@ -3152,13 +3115,13 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="34"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="19" t="s">
+      <c r="A19" s="42"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="45" t="s">
         <v>240</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="44" t="s">
         <v>70</v>
       </c>
       <c r="F19" s="46" t="s">
@@ -3167,6 +3130,16 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="C18:C19"/>
@@ -3176,62 +3149,30 @@
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
     <mergeCell ref="B12:B14"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C12:C14"/>
     <mergeCell ref="C16:C17"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="E2">
-    <cfRule type="containsText" dxfId="11" priority="10" stopIfTrue="1" operator="containsText" text="Hold">
+    <cfRule type="containsText" dxfId="5" priority="10" stopIfTrue="1" operator="containsText" text="Hold">
       <formula>NOT(ISERROR(SEARCH("Hold",E2)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="11" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="11" stopIfTrue="1" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="12" stopIfTrue="1" operator="containsText" text="Passed">
+    <cfRule type="containsText" dxfId="3" priority="12" stopIfTrue="1" operator="containsText" text="Passed">
       <formula>NOT(ISERROR(SEARCH("Passed",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E4">
-    <cfRule type="containsText" dxfId="8" priority="7" stopIfTrue="1" operator="containsText" text="Hold">
+  <conditionalFormatting sqref="E4:E17">
+    <cfRule type="containsText" dxfId="2" priority="1" stopIfTrue="1" operator="containsText" text="Hold">
       <formula>NOT(ISERROR(SEARCH("Hold",E4)))</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" stopIfTrue="1" operator="equal">
-      <formula>"Failed"</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="9" stopIfTrue="1" operator="containsText" text="Passed">
-      <formula>NOT(ISERROR(SEARCH("Passed",E4)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5">
-    <cfRule type="containsText" dxfId="5" priority="4" stopIfTrue="1" operator="containsText" text="Hold">
-      <formula>NOT(ISERROR(SEARCH("Hold",E5)))</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" stopIfTrue="1" operator="equal">
-      <formula>"Failed"</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="6" stopIfTrue="1" operator="containsText" text="Passed">
-      <formula>NOT(ISERROR(SEARCH("Passed",E5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E17">
-    <cfRule type="containsText" dxfId="2" priority="1" stopIfTrue="1" operator="containsText" text="Hold">
-      <formula>NOT(ISERROR(SEARCH("Hold",E6)))</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="3" stopIfTrue="1" operator="containsText" text="Passed">
-      <formula>NOT(ISERROR(SEARCH("Passed",E6)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Passed",E4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -3260,73 +3201,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="31" x14ac:dyDescent="0.7">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="43" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
     </row>
     <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="41" t="s">
         <v>222</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="41" t="s">
         <v>224</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="41" t="s">
         <v>226</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="F2" s="41" t="s">
         <v>227</v>
       </c>
-      <c r="G2" s="44" t="s">
+      <c r="G2" s="41" t="s">
         <v>228</v>
       </c>
-      <c r="H2" s="44" t="s">
+      <c r="H2" s="41" t="s">
         <v>229</v>
       </c>
-      <c r="I2" s="44" t="s">
+      <c r="I2" s="41" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="38" t="s">
         <v>231</v>
       </c>
       <c r="B3" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="C3" s="41">
+      <c r="C3" s="38">
         <v>18</v>
       </c>
-      <c r="D3" s="41">
+      <c r="D3" s="38">
         <v>15</v>
       </c>
-      <c r="E3" s="41">
+      <c r="E3" s="38">
         <v>3</v>
       </c>
-      <c r="F3" s="41">
+      <c r="F3" s="38">
         <v>18</v>
       </c>
-      <c r="G3" s="42">
+      <c r="G3" s="39">
         <v>0.83330000000000004</v>
       </c>
-      <c r="H3" s="42">
+      <c r="H3" s="39">
         <v>0.16669999999999999</v>
       </c>
-      <c r="I3" s="43">
+      <c r="I3" s="40">
         <v>1</v>
       </c>
     </row>

</xml_diff>